<commit_message>
Updated framework: Docker with selenium grid
</commit_message>
<xml_diff>
--- a/USA_State.xlsx
+++ b/USA_State.xlsx
@@ -4,11 +4,11 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13152" activeTab="2"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13152" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="NorthEast" sheetId="2" r:id="rId2"/>
+    <sheet name="Middle" sheetId="2" r:id="rId2"/>
     <sheet name="East" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="124519"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="114">
   <si>
     <t>Alabama</t>
   </si>
@@ -348,16 +348,16 @@
     <t>State</t>
   </si>
   <si>
-    <t xml:space="preserve"> Massachusetts</t>
-  </si>
-  <si>
     <t xml:space="preserve"> New Jersey</t>
   </si>
   <si>
-    <t xml:space="preserve"> New York</t>
-  </si>
-  <si>
     <t xml:space="preserve">  Pennsylvania </t>
+  </si>
+  <si>
+    <t>NorthEast</t>
+  </si>
+  <si>
+    <t>NewEngland</t>
   </si>
 </sst>
 </file>
@@ -1228,12 +1228,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>42</v>
+        <v>109</v>
       </c>
       <c r="B1" t="s">
         <v>43</v>
@@ -1241,58 +1241,18 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>111</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>110</v>
+        <v>86</v>
       </c>
       <c r="B3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2">
-      <c r="A4" t="s">
-        <v>72</v>
-      </c>
-      <c r="B4" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2">
-      <c r="A5" t="s">
-        <v>74</v>
-      </c>
-      <c r="B5" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2">
-      <c r="A6" t="s">
-        <v>111</v>
-      </c>
-      <c r="B6" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2">
-      <c r="A7" t="s">
-        <v>112</v>
-      </c>
-      <c r="B7" t="s">
         <v>87</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2">
-      <c r="A8" t="s">
-        <v>113</v>
-      </c>
-      <c r="B8" t="s">
-        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -1302,23 +1262,55 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>74</v>
+        <v>112</v>
       </c>
       <c r="B1" t="s">
-        <v>75</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B2" t="s">
         <v>79</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>74</v>
+      </c>
+      <c r="B3" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>